<commit_message>
updating low-biomass longread template and adding shortread template
</commit_message>
<xml_diff>
--- a/Assay_Templates/Omics_Assay_Templates/metagenome_seq_low-biomass_longreadDNAseq_w_GL-processed-data.xlsx
+++ b/Assay_Templates/Omics_Assay_Templates/metagenome_seq_low-biomass_longreadDNAseq_w_GL-processed-data.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/asaravia/Desktop/Logyx_NASA/GeneLab/Collaborations/JPL_PP/Test_Datasets/OSDR_Metadata_Templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/asaravia/Desktop/Logyx_NASA/GeneLab/Collaborations/JPL_PP/Test_Datasets/OSDR_Metadata_Templates/low-biomass_long-read_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDE54433-752A-0549-AD51-C1A1415A4E1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD99E82B-55BD-5B4E-9698-D62787A1FB29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35560" yWindow="500" windowWidth="37120" windowHeight="19540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="19540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191028"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="155">
   <si>
     <t>Metagenomics low-biomass long read DNA Seq table describes how the assay was performed - from Nucleic Acid Extraction to data generation</t>
   </si>
@@ -213,42 +212,12 @@
     <t>GeneLab metagenomics-lowbiomass-longread data processing protocol</t>
   </si>
   <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample1_raw_NanoPlot-report_GLlbnMetag.html</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample2_raw_NanoPlot-report_GLlbnMetag.html</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample3_raw_NanoPlot-report_GLlbnMetag.html</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample4_raw_NanoPlot-report_GLlbnMetag.html</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_raw_multiqc_data_GLlbnMetag.zip,GLDS-XXX_metagenomics-lowbiomass-longread_raw_multiqc_GLlbnMetag.html</t>
-  </si>
-  <si>
     <t>Filtered Sequence Data/NanoPlots</t>
   </si>
   <si>
     <t>Filtered Sequence Data/MultiQC Reports</t>
   </si>
   <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample1_filtered_NanoPlot-report_GLlbnMetag.html</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_filtered_multiqc_data_GLlbnMetag.zip,GLDS-XXX_metagenomics-lowbiomass-longread_filtered_multiqc_GLlbnMetag.html</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample2_filtered_NanoPlot-report_GLlbnMetag.html</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample3_filtered_NanoPlot-report_GLlbnMetag.html</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample4_filtered_NanoPlot-report_GLlbnMetag.html</t>
-  </si>
-  <si>
     <t>HR-removed Sequence Data/NanoPlots</t>
   </si>
   <si>
@@ -258,69 +227,12 @@
     <t>HR-removed Sequence Data/MultiQC Reports</t>
   </si>
   <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample1_HRrm_GLlbnMetag.fastq.gz</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample2_HRrm_GLlbnMetag.fastq.gz</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample3_HRrm_GLlbnMetag.fastq.gz</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample4_HRrm_GLlbnMetag.fastq.gz</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample1_HRrm_NanoPlot-report_GLlbnMetag.html</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_HRrm_multiqc_data_GLlbnMetag.zip,GLDS-XXX_metagenomics-lowbiomass-longread_HRrm_multiqc_GLlbnMetag.html</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample2_HRrm_NanoPlot-report_GLlbnMetag.html</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample3_HRrm_NanoPlot-report_GLlbnMetag.html</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample4_HRrm_NanoPlot-report_GLlbnMetag.html</t>
-  </si>
-  <si>
-    <t>Trimmed Sequence Data</t>
-  </si>
-  <si>
     <t>Trimmed Sequence Data/NanoPlots</t>
   </si>
   <si>
     <t>Trimmed Sequence Data/MultiQC Reports</t>
   </si>
   <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample1_trimmed_GLlbnMetag.fastq.gz</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample1_trimmed_NanoPlot-report_GLlbnMetag.html</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_trimmed_multiqc_data_GLlbnMetag.zip,GLDS-XXX_metagenomics-lowbiomass-longread_trimmed_multiqc_GLlbnMetag.html</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample2_trimmed_GLlbnMetag.fastq.gz</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample2_trimmed_NanoPlot-report_GLlbnMetag.html</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample3_trimmed_GLlbnMetag.fastq.gz</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample3_trimmed_NanoPlot-report_GLlbnMetag.html</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample4_trimmed_GLlbnMetag.fastq.gz</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample4_trimmed_NanoPlot-report_GLlbnMetag.html</t>
-  </si>
-  <si>
     <t>Decontaminated Sequence Data</t>
   </si>
   <si>
@@ -330,54 +242,12 @@
     <t>Decontaminated Sequence Data/MultiQC Reports</t>
   </si>
   <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample1_decontam_GLlbnMetag.fastq.gz</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample1_decontam_NanoPlot-report_GLlbnMetag.html</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_decontam_multiqc_data_GLlbnMetag.zip,GLDS-XXX_metagenomics-lowbiomass-longread_decontam_multiqc_GLlbnMetag.html</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample2_decontam_GLlbnMetag.fastq.gz</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample2_decontam_NanoPlot-report_GLlbnMetag.html</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample3_decontam_GLlbnMetag.fastq.gz</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample3_decontam_NanoPlot-report_GLlbnMetag.html</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample4_decontam_GLlbnMetag.fastq.gz</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample4_decontam_NanoPlot-report_GLlbnMetag.html</t>
-  </si>
-  <si>
     <t>Read-based Processing/Kaiju Outputs/Counts Tables</t>
   </si>
   <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_kaiju_raw_taxon_counts_GLlbnMetag.tsv,GLDS-XXX_metagenomics-lowbiomass-longread_kaiju_filtered_taxon_counts_GLlbnMetag.tsv,GLDS-XXX_metagenomics-lowbiomass-longread_kaiju_decontam_taxon_counts_GLlbnMetag.tsv</t>
-  </si>
-  <si>
-    <t>Read-based Processing/Kaiju Outputs/HTML Reports</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_kaiju_krona_report_GLlbnMetag.html,GLDS-XXX_metagenomics-lowbiomass-longread_kaiju_combined_report_GLlbnMetag.html</t>
-  </si>
-  <si>
     <t>Read-based Processing/Kraken2 Outputs/Counts Tables</t>
   </si>
   <si>
-    <t>Read-based Processing/Kraken2 Outputs/HTML Reports</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_kraken2_krona_report_GLlbnMetag.html,GLDS-XXX_metagenomics-lowbiomass-longread_kraken2_combined_report_GLlbnMetag.html</t>
-  </si>
-  <si>
     <t>Assembly-based Processing</t>
   </si>
   <si>
@@ -393,121 +263,247 @@
     <t>Assembly-based Processing/MAGs</t>
   </si>
   <si>
-    <t>Assembly-based Processing/combined-outputs</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_Assembly-based-processing-overview_GLlbnMetag.tsv</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample1_assembly_GLlbnMetag.fasta,GLDS-XXX_metagenomics-lowbiomass-longread_assembly-summaries_GLlbnMetag.tsv</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample2_assembly_GLlbnMetag.fasta,GLDS-XXX_metagenomics-lowbiomass-longread_assembly-summaries_GLlbnMetag.tsv</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample3_assembly_GLlbnMetag.fasta,GLDS-XXX_metagenomics-lowbiomass-longread_assembly-summaries_GLlbnMetag.tsv</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample4_assembly_GLlbnMetag.fasta,GLDS-XXX_metagenomics-lowbiomass-longread_assembly-summaries_GLlbnMetag.tsv</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample1_genes_GLlbnMetag.fasta,GLDS-XXX_metagenomics-lowbiomass-longread_sample1_genes_GLlbnMetag.faa,GLDS-XXX_metagenomics-lowbiomass-longread_sample1_genes_GLlbnMetag.gff</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample2_genes_GLlbnMetag.fasta,GLDS-XXX_metagenomics-lowbiomass-longread_sample2_genes_GLlbnMetag.faa,GLDS-XXX_metagenomics-lowbiomass-longread_sample2_genes_GLlbnMetag.gff</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample3_genes_GLlbnMetag.fasta,GLDS-XXX_metagenomics-lowbiomass-longread_sample3_genes_GLlbnMetag.faa,GLDS-XXX_metagenomics-lowbiomass-longread_sample3_genes_GLlbnMetag.gff</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample4_genes_GLlbnMetag.fasta,GLDS-XXX_metagenomics-lowbiomass-longread_sample4_genes_GLlbnMetag.faa,GLDS-XXX_metagenomics-lowbiomass-longread_sample4_genes_GLlbnMetag.gff</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample1_gene-coverage-annotation-and-tax_GLlbnMetag.tsv,GLDS-XXX_metagenomics-lowbiomass-longread_sample1_contig-coverage-and-tax_GLlbnMetag.tsv</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample2_gene-coverage-annotation-and-tax_GLlbnMetag.tsv,GLDS-XXX_metagenomics-lowbiomass-longread_sample2_contig-coverage-and-tax_GLlbnMetag.tsv</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample3_gene-coverage-annotation-and-tax_GLlbnMetag.tsv,GLDS-XXX_metagenomics-lowbiomass-longread_sample3_contig-coverage-and-tax_GLlbnMetag.tsv</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample4_gene-coverage-annotation-and-tax_GLlbnMetag.tsv,GLDS-XXX_metagenomics-lowbiomass-longread_sample4_contig-coverage-and-tax_GLlbnMetag.tsv</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample1_GLlbnMetag.bam,GLDS-XXX_metagenomics-lowbiomass-longread_sample1_mapping-info_GLlbnMetag.txt,GLDS-XXX_metagenomics-lowbiomass-longread_sample1_metabat-assembly-depth_GLlbnMetag.tsv</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample2_GLlbnMetag.bam,GLDS-XXX_metagenomics-lowbiomass-longread_sample2_mapping-info_GLlbnMetag.txt,GLDS-XXX_metagenomics-lowbiomass-longread_sample2_metabat-assembly-depth_GLlbnMetag.tsv</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample3_GLlbnMetag.bam,GLDS-XXX_metagenomics-lowbiomass-longread_sample3_mapping-info_GLlbnMetag.txt,GLDS-XXX_metagenomics-lowbiomass-longread_sample3_metabat-assembly-depth_GLlbnMetag.tsv</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample4_GLlbnMetag.bam,GLDS-XXX_metagenomics-lowbiomass-longread_sample4_mapping-info_GLlbnMetag.txt,GLDS-XXX_metagenomics-lowbiomass-longread_sample4_metabat-assembly-depth_GLlbnMetag.tsv</t>
-  </si>
-  <si>
     <t>Assembly-based Processing/read-mapping</t>
   </si>
   <si>
     <t>Assembly-based Processing/bins</t>
   </si>
   <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample1_bins_GLlbnMetag.zip,GLDS-XXX_metagenomics-lowbiomass-longread_bins-overview_GLlbnMetag.tsv</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample2_bins_GLlbnMetag.zip,GLDS-XXX_metagenomics-lowbiomass-longread_bins-overview_GLlbnMetag.tsv</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample3_bins_GLlbnMetag.zip,GLDS-XXX_metagenomics-lowbiomass-longread_bins-overview_GLlbnMetag.tsv</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample4_bins_GLlbnMetag.zip,GLDS-XXX_metagenomics-lowbiomass-longread_bins-overview_GLlbnMetag.tsv</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_kaiju_NoFilter_taxon_counts_GLlbnMetag.tsv,GLDS-XXX_metagenomics-lowbiomass-longread_kaiju_filtered_taxon_counts_GLlbnMetag.tsv,GLDS-XXX_metagenomics-lowbiomass-longread_kaiju_decontam_taxon_counts_GLlbnMetag.tsv</t>
-  </si>
-  <si>
     <t>Merged Sequence Data/NanoPlots</t>
   </si>
   <si>
     <t>Merged Sequence Data/MultiQC Reports</t>
   </si>
   <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample1_MAGs_GLlbnMetag.zip,GLDS-XXX_metagenomics-lowbiomass-longread_MAGs-overview_GLlbnMetag.tsv</t>
-  </si>
-  <si>
     <t>Assembly-based Processing/MAGs/KEGG_Outputs</t>
   </si>
   <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_MAG-KEGG-Decoder-out_GLlbnMetag.tsv,GLDS-XXX_metagenomics-lowbiomass-longread_MAG-KEGG-Decoder-out_GLlbnMetag.html,GLDS-XXX_metagenomics-lowbiomass-longread_MAG-level-KO-annotations_GLlbnMetag.tsv</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_assembly_combined_report_GLlbnMetag.html</t>
-  </si>
-  <si>
     <t>Assembly-based Processing/combined-outputs/Gene-level/Taxonomy</t>
   </si>
   <si>
     <t>Assembly-based Processing/combined-outputs/Contig-level</t>
   </si>
   <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_Combined-contig-level-taxonomy-coverages-CPM_GLlbnMetag.tsv,GLDS-XXX_metagenomics-lowbiomass-longread_Combined-contig-level-taxonomy-coverages_GLlbnMetag.tsv</t>
-  </si>
-  <si>
     <t>Assembly-based Processing/combined-outputs/Gene-level/KO</t>
   </si>
   <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_Combined-gene-level-taxonomy-coverages-CPM_GLlbnMetag.tsv,GLDS-XXX_metagenomics-lowbiomass-longread_Combined-gene-level-taxonomy-coverages_GLlbnMetag.tsv</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_Combined-gene-level-KO-function-coverages-CPM_GLlbnMetag.tsv,GLDS-XXX_metagenomics-lowbiomass-longread_Combined-gene-level-KO-function-coverages_GLlbnMetag.tsv</t>
-  </si>
-  <si>
-    <t>GLDS-XXX_metagenomics-lowbiomass-longread_kraken2_NoFilter_taxon_counts_GLlbnMetag.tsv,GLDS-XXX_metagenomics-lowbiomass-longread_kraken2_filtered_taxon_counts_GLlbnMetag.tsv,GLDS-XXX_metagenomics-lowbiomass-longread_kraken2_decontam_taxon_counts_GLlbnMetag.tsv</t>
-  </si>
-  <si>
     <t>Contaminant Reads Removed</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample1_raw_NanoPlot-report_GLlblMetag.html</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_raw_multiqc_data_GLlblMetag.zip,GLDS-XXX_metagenomics-lowbiomass-longread_raw_multiqc_GLlblMetag.html</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample1_filtered_NanoPlot-report_GLlblMetag.html</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_filtered_multiqc_data_GLlblMetag.zip,GLDS-XXX_metagenomics-lowbiomass-longread_filtered_multiqc_GLlblMetag.html</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample1_trimmed_NanoPlot-report_GLlblMetag.html</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_trimmed_multiqc_data_GLlblMetag.zip,GLDS-XXX_metagenomics-lowbiomass-longread_trimmed_multiqc_GLlblMetag.html</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample1_HRrm_GLlblMetag.fastq.gz</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample1_HRrm_NanoPlot-report_GLlblMetag.html</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_HRrm_multiqc_data_GLlblMetag.zip,GLDS-XXX_metagenomics-lowbiomass-longread_HRrm_multiqc_GLlblMetag.html</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample1_decontam_GLlblMetag.fastq.gz</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample1_decontam_NanoPlot-report_GLlblMetag.html</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_decontam_multiqc_data_GLlblMetag.zip,GLDS-XXX_metagenomics-lowbiomass-longread_decontam_multiqc_GLlblMetag.html</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_kaiju_NoFilter_taxon_counts_GLlblMetag.tsv,GLDS-XXX_metagenomics-lowbiomass-longread_kaiju_filtered_taxon_counts_GLlblMetag.tsv,GLDS-XXX_metagenomics-lowbiomass-longread_kaiju_decontam_taxon_counts_GLlblMetag.tsv</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_kraken2_NoFilter_taxon_counts_GLlblMetag.tsv,GLDS-XXX_metagenomics-lowbiomass-longread_kraken2_filtered_taxon_counts_GLlblMetag.tsv,GLDS-XXX_metagenomics-lowbiomass-longread_kraken2_decontam_taxon_counts_GLlblMetag.tsv</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_Assembly-based-processing-overview_GLlblMetag.tsv</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample1_assembly_GLlblMetag.fasta,GLDS-XXX_metagenomics-lowbiomass-longread_assembly-summaries_GLlblMetag.tsv</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample1_genes_GLlblMetag.fasta,GLDS-XXX_metagenomics-lowbiomass-longread_sample1_genes_GLlblMetag.faa,GLDS-XXX_metagenomics-lowbiomass-longread_sample1_genes_GLlblMetag.gff</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample1_gene-coverage-annotation-and-tax_GLlblMetag.tsv,GLDS-XXX_metagenomics-lowbiomass-longread_sample1_contig-coverage-and-tax_GLlblMetag.tsv</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample1_GLlblMetag.bam,GLDS-XXX_metagenomics-lowbiomass-longread_sample1_mapping-info_GLlblMetag.txt,GLDS-XXX_metagenomics-lowbiomass-longread_sample1_metabat-assembly-depth_GLlblMetag.tsv</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample1_bins_GLlblMetag.zip,GLDS-XXX_metagenomics-lowbiomass-longread_bins-overview_GLlblMetag.tsv</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample1_MAGs_GLlblMetag.zip,GLDS-XXX_metagenomics-lowbiomass-longread_MAGs-overview_GLlblMetag.tsv</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_MAG-KEGG-Decoder-out_GLlblMetag.tsv,GLDS-XXX_metagenomics-lowbiomass-longread_MAG-KEGG-Decoder-out_GLlblMetag.html,GLDS-XXX_metagenomics-lowbiomass-longread_MAG-level-KO-annotations_GLlblMetag.tsv</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample2_raw_NanoPlot-report_GLlblMetag.html</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample2_filtered_NanoPlot-report_GLlblMetag.html</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample2_trimmed_NanoPlot-report_GLlblMetag.html</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample2_HRrm_GLlblMetag.fastq.gz</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample2_HRrm_NanoPlot-report_GLlblMetag.html</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample2_decontam_GLlblMetag.fastq.gz</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample2_decontam_NanoPlot-report_GLlblMetag.html</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample2_assembly_GLlblMetag.fasta,GLDS-XXX_metagenomics-lowbiomass-longread_assembly-summaries_GLlblMetag.tsv</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample2_genes_GLlblMetag.fasta,GLDS-XXX_metagenomics-lowbiomass-longread_sample2_genes_GLlblMetag.faa,GLDS-XXX_metagenomics-lowbiomass-longread_sample2_genes_GLlblMetag.gff</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample2_gene-coverage-annotation-and-tax_GLlblMetag.tsv,GLDS-XXX_metagenomics-lowbiomass-longread_sample2_contig-coverage-and-tax_GLlblMetag.tsv</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample2_GLlblMetag.bam,GLDS-XXX_metagenomics-lowbiomass-longread_sample2_mapping-info_GLlblMetag.txt,GLDS-XXX_metagenomics-lowbiomass-longread_sample2_metabat-assembly-depth_GLlblMetag.tsv</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample2_bins_GLlblMetag.zip,GLDS-XXX_metagenomics-lowbiomass-longread_bins-overview_GLlblMetag.tsv</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample3_raw_NanoPlot-report_GLlblMetag.html</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample3_filtered_NanoPlot-report_GLlblMetag.html</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample3_trimmed_NanoPlot-report_GLlblMetag.html</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample3_HRrm_GLlblMetag.fastq.gz</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample3_HRrm_NanoPlot-report_GLlblMetag.html</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample3_decontam_GLlblMetag.fastq.gz</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample3_decontam_NanoPlot-report_GLlblMetag.html</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample3_assembly_GLlblMetag.fasta,GLDS-XXX_metagenomics-lowbiomass-longread_assembly-summaries_GLlblMetag.tsv</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample3_genes_GLlblMetag.fasta,GLDS-XXX_metagenomics-lowbiomass-longread_sample3_genes_GLlblMetag.faa,GLDS-XXX_metagenomics-lowbiomass-longread_sample3_genes_GLlblMetag.gff</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample3_gene-coverage-annotation-and-tax_GLlblMetag.tsv,GLDS-XXX_metagenomics-lowbiomass-longread_sample3_contig-coverage-and-tax_GLlblMetag.tsv</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample3_GLlblMetag.bam,GLDS-XXX_metagenomics-lowbiomass-longread_sample3_mapping-info_GLlblMetag.txt,GLDS-XXX_metagenomics-lowbiomass-longread_sample3_metabat-assembly-depth_GLlblMetag.tsv</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample3_bins_GLlblMetag.zip,GLDS-XXX_metagenomics-lowbiomass-longread_bins-overview_GLlblMetag.tsv</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample4_raw_NanoPlot-report_GLlblMetag.html</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample4_filtered_NanoPlot-report_GLlblMetag.html</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample4_trimmed_NanoPlot-report_GLlblMetag.html</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample4_HRrm_GLlblMetag.fastq.gz</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample4_HRrm_NanoPlot-report_GLlblMetag.html</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample4_decontam_GLlblMetag.fastq.gz</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample4_decontam_NanoPlot-report_GLlblMetag.html</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample4_assembly_GLlblMetag.fasta,GLDS-XXX_metagenomics-lowbiomass-longread_assembly-summaries_GLlblMetag.tsv</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample4_genes_GLlblMetag.fasta,GLDS-XXX_metagenomics-lowbiomass-longread_sample4_genes_GLlblMetag.faa,GLDS-XXX_metagenomics-lowbiomass-longread_sample4_genes_GLlblMetag.gff</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample4_gene-coverage-annotation-and-tax_GLlblMetag.tsv,GLDS-XXX_metagenomics-lowbiomass-longread_sample4_contig-coverage-and-tax_GLlblMetag.tsv</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample4_GLlblMetag.bam,GLDS-XXX_metagenomics-lowbiomass-longread_sample4_mapping-info_GLlblMetag.txt,GLDS-XXX_metagenomics-lowbiomass-longread_sample4_metabat-assembly-depth_GLlblMetag.tsv</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample4_bins_GLlblMetag.zip,GLDS-XXX_metagenomics-lowbiomass-longread_bins-overview_GLlblMetag.tsv</t>
+  </si>
+  <si>
+    <t>Read-based Processing/Kaiju Outputs/Barplots</t>
+  </si>
+  <si>
+    <t>Read-based Processing/Kaiju Outputs/Krona Reports</t>
+  </si>
+  <si>
+    <t>Read-based Processing/Kraken2 Outputs/Barplots</t>
+  </si>
+  <si>
+    <t>Read-based Processing/Kraken2 Outputs/Krona Reports</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample2_MAGs_GLlblMetag.zip,GLDS-XXX_metagenomics-lowbiomass-longread_MAGs-overview_GLlblMetag.tsv</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample3_MAGs_GLlblMetag.zip,GLDS-XXX_metagenomics-lowbiomass-longread_MAGs-overview_GLlblMetag.tsv</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_sample4_MAGs_GLlblMetag.zip,GLDS-XXX_metagenomics-lowbiomass-longread_MAGs-overview_GLlblMetag.tsv</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_kaiju_unfiltered_species_barplot_GLlblMetag.html,GLDS-XXX_metagenomics-lowbiomass-longread_kaiju_filtered_species_barplot_GLlblMetag.html,GLDS-XXX_metagenomics-lowbiomass-longread_kaiju_decontam_species_barplot_GLlblMetag.html</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_kaiju_krona_report_GLlblMetag.html</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_kraken2_unfiltered_species_barplot_GLlblMetag.html,GLDS-XXX_metagenomics-lowbiomass-longread_kraken2_filtered_species_barplot_GLlblMetag.html,GLDS-XXX_metagenomics-lowbiomass-longread_kraken2_decontam_species_barplot_GLlblMetag.html</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_kraken2_krona_report_GLlblMetag.html</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_Combined-gene-level-taxonomy-coverages-CPM_GLlblMetag.tsv,GLDS-XXX_metagenomics-lowbiomass-longread_Combined-gene-level-taxonomy-coverages_GLlblMetag.tsv,GLDS-XXX_metagenomics-lowbiomass-longread_Combined-gene-level-taxonomy-heatmap_GLlblMetag.png</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_Combined-gene-level-KO-function-coverages-CPM_GLlblMetag.tsv,GLDS-XXX_metagenomics-lowbiomass-longread_Combined-gene-level-KO-function-coverages_GLlblMetag.tsv,GLDS-XXX_metagenomics-lowbiomass-longread_Combined-gene-level-KO-function-heatmap_GLlblMetag.png</t>
+  </si>
+  <si>
+    <t>GLDS-XXX_metagenomics-lowbiomass-longread_Combined-contig-level-taxonomy-coverages-CPM_GLlblMetag.tsv,GLDS-XXX_metagenomics-lowbiomass-longread_Combined-contig-level-taxonomy-coverages_GLlblMetag.tsv,GLDS-XXX_metagenomics-lowbiomass-longread_Combined-contig-level-taxonomy-heatmap_GLlblMetag.png</t>
   </si>
 </sst>
 </file>
@@ -554,7 +550,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -627,11 +623,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -665,6 +676,13 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -896,7 +914,11 @@
     <col min="23" max="26" width="11.5" customWidth="1"/>
     <col min="27" max="27" width="17" customWidth="1"/>
     <col min="28" max="28" width="16.1640625" customWidth="1"/>
-    <col min="29" max="59" width="11.5" customWidth="1"/>
+    <col min="29" max="43" width="11.5" customWidth="1"/>
+    <col min="44" max="45" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="11.5" customWidth="1"/>
+    <col min="47" max="48" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="49" max="59" width="11.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:59" x14ac:dyDescent="0.2">
@@ -998,94 +1020,94 @@
         <v>3</v>
       </c>
       <c r="AD3" s="3" t="s">
-        <v>155</v>
+        <v>82</v>
       </c>
       <c r="AE3" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="AF3" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="AG3" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="AH3" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AI3" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="AJ3" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="AK3" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AL3" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="AM3" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="AN3" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="AO3" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="AP3" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="AQ3" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="AR3" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="AS3" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="AF3" s="3" t="s">
+      <c r="AT3" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="AU3" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="AG3" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="AH3" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="AI3" s="3" t="s">
+      <c r="AV3" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="AW3" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="AX3" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="AJ3" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="AK3" s="3" t="s">
+      <c r="AY3" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="AL3" s="3" t="s">
+      <c r="AZ3" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="BA3" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="BB3" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="BC3" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="BD3" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="BE3" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="BF3" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="AM3" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="AN3" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="AO3" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="AP3" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="AQ3" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="AR3" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="AS3" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="AT3" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="AU3" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="AV3" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="AW3" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="AX3" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="AY3" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="AZ3" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="BA3" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="BB3" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="BC3" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="BD3" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="BE3" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="BF3" s="3" t="s">
-        <v>151</v>
-      </c>
       <c r="BG3" s="3" t="s">
-        <v>149</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:59" ht="112" x14ac:dyDescent="0.2">
@@ -1182,11 +1204,11 @@
       <c r="AO4" s="5"/>
       <c r="AP4" s="5"/>
       <c r="AQ4" s="5"/>
-      <c r="AR4" s="5"/>
-      <c r="AS4" s="5"/>
+      <c r="AR4" s="17"/>
+      <c r="AS4" s="17"/>
       <c r="AT4" s="5"/>
-      <c r="AU4" s="5"/>
-      <c r="AV4" s="5"/>
+      <c r="AU4" s="17"/>
+      <c r="AV4" s="17"/>
       <c r="AW4" s="5"/>
       <c r="AX4" s="5"/>
       <c r="AY4" s="5"/>
@@ -1245,82 +1267,82 @@
       </c>
       <c r="AD5" s="9"/>
       <c r="AE5" s="9" t="s">
-        <v>57</v>
+        <v>83</v>
       </c>
       <c r="AF5" s="9" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="AG5" s="9" t="s">
-        <v>64</v>
+        <v>85</v>
       </c>
       <c r="AH5" s="9" t="s">
-        <v>65</v>
+        <v>86</v>
       </c>
       <c r="AI5" s="9" t="s">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="AJ5" s="9" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="AK5" s="9" t="s">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="AL5" s="9" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="AM5" s="9" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="AN5" s="9" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="AO5" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="AP5" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="AQ5" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="AR5" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="AS5" s="18" t="s">
+        <v>149</v>
+      </c>
+      <c r="AT5" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="AP5" s="9" t="s">
+      <c r="AU5" s="18" t="s">
+        <v>150</v>
+      </c>
+      <c r="AV5" s="18" t="s">
+        <v>151</v>
+      </c>
+      <c r="AW5" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="AQ5" s="9" t="s">
+      <c r="AX5" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="AR5" s="9" t="s">
-        <v>141</v>
-      </c>
-      <c r="AS5" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="AT5" s="9" t="s">
-        <v>154</v>
-      </c>
-      <c r="AU5" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="AV5" s="9" t="s">
-        <v>118</v>
-      </c>
-      <c r="AW5" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="AX5" s="9" t="s">
-        <v>123</v>
-      </c>
       <c r="AY5" s="9" t="s">
-        <v>127</v>
+        <v>99</v>
       </c>
       <c r="AZ5" s="9" t="s">
-        <v>131</v>
+        <v>100</v>
       </c>
       <c r="BA5" s="9" t="s">
-        <v>137</v>
+        <v>101</v>
       </c>
       <c r="BB5" s="9" t="s">
-        <v>144</v>
+        <v>102</v>
       </c>
       <c r="BC5" s="9" t="s">
-        <v>146</v>
+        <v>103</v>
       </c>
       <c r="BD5" s="9" t="s">
-        <v>147</v>
+        <v>104</v>
       </c>
       <c r="BE5" s="9" t="s">
         <v>152</v>
@@ -1329,7 +1351,7 @@
         <v>153</v>
       </c>
       <c r="BG5" s="9" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="6" spans="1:59" ht="409.6" x14ac:dyDescent="0.2">
@@ -1368,82 +1390,82 @@
       <c r="AC6" s="15"/>
       <c r="AD6" s="12"/>
       <c r="AE6" s="9" t="s">
-        <v>58</v>
+        <v>105</v>
       </c>
       <c r="AF6" s="9" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="AG6" s="9" t="s">
-        <v>66</v>
+        <v>106</v>
       </c>
       <c r="AH6" s="9" t="s">
-        <v>65</v>
+        <v>86</v>
       </c>
       <c r="AI6" s="9" t="s">
-        <v>73</v>
+        <v>107</v>
       </c>
       <c r="AJ6" s="9" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="AK6" s="9" t="s">
-        <v>77</v>
+        <v>108</v>
       </c>
       <c r="AL6" s="9" t="s">
-        <v>87</v>
+        <v>109</v>
       </c>
       <c r="AM6" s="9" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="AN6" s="9" t="s">
-        <v>86</v>
+        <v>110</v>
       </c>
       <c r="AO6" s="9" t="s">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="AP6" s="9" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="AQ6" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="AR6" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="AS6" s="9" t="s">
-        <v>108</v>
+        <v>95</v>
+      </c>
+      <c r="AR6" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="AS6" s="18" t="s">
+        <v>149</v>
       </c>
       <c r="AT6" s="9" t="s">
-        <v>154</v>
-      </c>
-      <c r="AU6" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="AV6" s="9" t="s">
-        <v>118</v>
+        <v>96</v>
+      </c>
+      <c r="AU6" s="18" t="s">
+        <v>150</v>
+      </c>
+      <c r="AV6" s="18" t="s">
+        <v>151</v>
       </c>
       <c r="AW6" s="9" t="s">
-        <v>120</v>
+        <v>97</v>
       </c>
       <c r="AX6" s="9" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="AY6" s="9" t="s">
-        <v>128</v>
+        <v>113</v>
       </c>
       <c r="AZ6" s="9" t="s">
-        <v>132</v>
+        <v>114</v>
       </c>
       <c r="BA6" s="9" t="s">
-        <v>138</v>
+        <v>115</v>
       </c>
       <c r="BB6" s="9" t="s">
-        <v>144</v>
+        <v>116</v>
       </c>
       <c r="BC6" s="9" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="BD6" s="9" t="s">
-        <v>147</v>
+        <v>104</v>
       </c>
       <c r="BE6" s="9" t="s">
         <v>152</v>
@@ -1452,7 +1474,7 @@
         <v>153</v>
       </c>
       <c r="BG6" s="9" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="7" spans="1:59" ht="409.6" x14ac:dyDescent="0.2">
@@ -1491,82 +1513,82 @@
       <c r="AC7" s="15"/>
       <c r="AD7" s="12"/>
       <c r="AE7" s="9" t="s">
-        <v>59</v>
+        <v>117</v>
       </c>
       <c r="AF7" s="9" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="AG7" s="9" t="s">
-        <v>67</v>
+        <v>118</v>
       </c>
       <c r="AH7" s="9" t="s">
-        <v>65</v>
+        <v>86</v>
       </c>
       <c r="AI7" s="9" t="s">
-        <v>74</v>
+        <v>119</v>
       </c>
       <c r="AJ7" s="9" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AK7" s="9" t="s">
-        <v>77</v>
+        <v>120</v>
       </c>
       <c r="AL7" s="9" t="s">
-        <v>89</v>
+        <v>121</v>
       </c>
       <c r="AM7" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="AN7" s="9" t="s">
-        <v>86</v>
+        <v>122</v>
       </c>
       <c r="AO7" s="9" t="s">
-        <v>101</v>
+        <v>123</v>
       </c>
       <c r="AP7" s="9" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="AQ7" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="AR7" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="AS7" s="9" t="s">
-        <v>108</v>
+        <v>95</v>
+      </c>
+      <c r="AR7" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="AS7" s="18" t="s">
+        <v>149</v>
       </c>
       <c r="AT7" s="9" t="s">
-        <v>154</v>
-      </c>
-      <c r="AU7" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="AV7" s="9" t="s">
-        <v>118</v>
+        <v>96</v>
+      </c>
+      <c r="AU7" s="18" t="s">
+        <v>150</v>
+      </c>
+      <c r="AV7" s="18" t="s">
+        <v>151</v>
       </c>
       <c r="AW7" s="9" t="s">
-        <v>121</v>
+        <v>97</v>
       </c>
       <c r="AX7" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="AY7" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="AY7" s="9" t="s">
-        <v>129</v>
-      </c>
       <c r="AZ7" s="9" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="BA7" s="9" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="BB7" s="9" t="s">
-        <v>144</v>
+        <v>128</v>
       </c>
       <c r="BC7" s="9" t="s">
         <v>146</v>
       </c>
       <c r="BD7" s="9" t="s">
-        <v>147</v>
+        <v>104</v>
       </c>
       <c r="BE7" s="9" t="s">
         <v>152</v>
@@ -1575,7 +1597,7 @@
         <v>153</v>
       </c>
       <c r="BG7" s="9" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="8" spans="1:59" ht="409.6" x14ac:dyDescent="0.2">
@@ -1614,82 +1636,82 @@
       <c r="AC8" s="15"/>
       <c r="AD8" s="12"/>
       <c r="AE8" s="9" t="s">
-        <v>60</v>
+        <v>129</v>
       </c>
       <c r="AF8" s="9" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="AG8" s="9" t="s">
-        <v>68</v>
+        <v>130</v>
       </c>
       <c r="AH8" s="9" t="s">
-        <v>65</v>
+        <v>86</v>
       </c>
       <c r="AI8" s="9" t="s">
-        <v>75</v>
+        <v>131</v>
       </c>
       <c r="AJ8" s="9" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="AK8" s="9" t="s">
-        <v>77</v>
+        <v>132</v>
       </c>
       <c r="AL8" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="AM8" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="AM8" s="9" t="s">
-        <v>92</v>
-      </c>
       <c r="AN8" s="9" t="s">
-        <v>86</v>
+        <v>134</v>
       </c>
       <c r="AO8" s="9" t="s">
-        <v>103</v>
+        <v>135</v>
       </c>
       <c r="AP8" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="AQ8" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="AR8" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="AS8" s="18" t="s">
+        <v>149</v>
+      </c>
+      <c r="AT8" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="AU8" s="18" t="s">
+        <v>150</v>
+      </c>
+      <c r="AV8" s="18" t="s">
+        <v>151</v>
+      </c>
+      <c r="AW8" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="AX8" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="AY8" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="AZ8" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="BA8" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="BB8" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="BC8" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="BD8" s="9" t="s">
         <v>104</v>
-      </c>
-      <c r="AQ8" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="AR8" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="AS8" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="AT8" s="9" t="s">
-        <v>154</v>
-      </c>
-      <c r="AU8" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="AV8" s="9" t="s">
-        <v>118</v>
-      </c>
-      <c r="AW8" s="9" t="s">
-        <v>122</v>
-      </c>
-      <c r="AX8" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="AY8" s="9" t="s">
-        <v>130</v>
-      </c>
-      <c r="AZ8" s="9" t="s">
-        <v>134</v>
-      </c>
-      <c r="BA8" s="9" t="s">
-        <v>140</v>
-      </c>
-      <c r="BB8" s="9" t="s">
-        <v>144</v>
-      </c>
-      <c r="BC8" s="9" t="s">
-        <v>146</v>
-      </c>
-      <c r="BD8" s="9" t="s">
-        <v>147</v>
       </c>
       <c r="BE8" s="9" t="s">
         <v>152</v>
@@ -1698,7 +1720,7 @@
         <v>153</v>
       </c>
       <c r="BG8" s="9" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="9" spans="1:59" x14ac:dyDescent="0.2">
@@ -1749,11 +1771,11 @@
       <c r="AO9" s="12"/>
       <c r="AP9" s="12"/>
       <c r="AQ9" s="12"/>
-      <c r="AR9" s="12"/>
-      <c r="AS9" s="12"/>
+      <c r="AR9" s="19"/>
+      <c r="AS9" s="19"/>
       <c r="AT9" s="12"/>
-      <c r="AU9" s="12"/>
-      <c r="AV9" s="12"/>
+      <c r="AU9" s="19"/>
+      <c r="AV9" s="19"/>
       <c r="AW9" s="12"/>
       <c r="AX9" s="12"/>
       <c r="AY9" s="12"/>
@@ -1814,11 +1836,11 @@
       <c r="AO10" s="12"/>
       <c r="AP10" s="12"/>
       <c r="AQ10" s="12"/>
-      <c r="AR10" s="12"/>
-      <c r="AS10" s="12"/>
+      <c r="AR10" s="19"/>
+      <c r="AS10" s="19"/>
       <c r="AT10" s="12"/>
-      <c r="AU10" s="12"/>
-      <c r="AV10" s="12"/>
+      <c r="AU10" s="19"/>
+      <c r="AV10" s="19"/>
       <c r="AW10" s="12"/>
       <c r="AX10" s="12"/>
       <c r="AY10" s="12"/>
@@ -1879,11 +1901,11 @@
       <c r="AO11" s="12"/>
       <c r="AP11" s="12"/>
       <c r="AQ11" s="12"/>
-      <c r="AR11" s="12"/>
-      <c r="AS11" s="12"/>
+      <c r="AR11" s="19"/>
+      <c r="AS11" s="19"/>
       <c r="AT11" s="12"/>
-      <c r="AU11" s="12"/>
-      <c r="AV11" s="12"/>
+      <c r="AU11" s="19"/>
+      <c r="AV11" s="19"/>
       <c r="AW11" s="12"/>
       <c r="AX11" s="12"/>
       <c r="AY11" s="12"/>
@@ -1944,11 +1966,11 @@
       <c r="AO12" s="12"/>
       <c r="AP12" s="12"/>
       <c r="AQ12" s="12"/>
-      <c r="AR12" s="12"/>
-      <c r="AS12" s="12"/>
+      <c r="AR12" s="19"/>
+      <c r="AS12" s="19"/>
       <c r="AT12" s="12"/>
-      <c r="AU12" s="12"/>
-      <c r="AV12" s="12"/>
+      <c r="AU12" s="19"/>
+      <c r="AV12" s="19"/>
       <c r="AW12" s="12"/>
       <c r="AX12" s="12"/>
       <c r="AY12" s="12"/>
@@ -2009,11 +2031,11 @@
       <c r="AO13" s="12"/>
       <c r="AP13" s="12"/>
       <c r="AQ13" s="12"/>
-      <c r="AR13" s="12"/>
-      <c r="AS13" s="12"/>
+      <c r="AR13" s="19"/>
+      <c r="AS13" s="19"/>
       <c r="AT13" s="12"/>
-      <c r="AU13" s="12"/>
-      <c r="AV13" s="12"/>
+      <c r="AU13" s="19"/>
+      <c r="AV13" s="19"/>
       <c r="AW13" s="12"/>
       <c r="AX13" s="12"/>
       <c r="AY13" s="12"/>
@@ -2074,11 +2096,11 @@
       <c r="AO14" s="12"/>
       <c r="AP14" s="12"/>
       <c r="AQ14" s="12"/>
-      <c r="AR14" s="12"/>
-      <c r="AS14" s="12"/>
+      <c r="AR14" s="19"/>
+      <c r="AS14" s="19"/>
       <c r="AT14" s="12"/>
-      <c r="AU14" s="12"/>
-      <c r="AV14" s="12"/>
+      <c r="AU14" s="19"/>
+      <c r="AV14" s="19"/>
       <c r="AW14" s="12"/>
       <c r="AX14" s="12"/>
       <c r="AY14" s="12"/>
@@ -2139,11 +2161,11 @@
       <c r="AO15" s="12"/>
       <c r="AP15" s="12"/>
       <c r="AQ15" s="12"/>
-      <c r="AR15" s="12"/>
-      <c r="AS15" s="12"/>
+      <c r="AR15" s="19"/>
+      <c r="AS15" s="19"/>
       <c r="AT15" s="12"/>
-      <c r="AU15" s="12"/>
-      <c r="AV15" s="12"/>
+      <c r="AU15" s="19"/>
+      <c r="AV15" s="19"/>
       <c r="AW15" s="12"/>
       <c r="AX15" s="12"/>
       <c r="AY15" s="12"/>
@@ -2204,11 +2226,11 @@
       <c r="AO16" s="12"/>
       <c r="AP16" s="12"/>
       <c r="AQ16" s="12"/>
-      <c r="AR16" s="12"/>
-      <c r="AS16" s="12"/>
+      <c r="AR16" s="19"/>
+      <c r="AS16" s="19"/>
       <c r="AT16" s="12"/>
-      <c r="AU16" s="12"/>
-      <c r="AV16" s="12"/>
+      <c r="AU16" s="19"/>
+      <c r="AV16" s="19"/>
       <c r="AW16" s="12"/>
       <c r="AX16" s="12"/>
       <c r="AY16" s="12"/>
@@ -2269,11 +2291,11 @@
       <c r="AO17" s="12"/>
       <c r="AP17" s="12"/>
       <c r="AQ17" s="12"/>
-      <c r="AR17" s="12"/>
-      <c r="AS17" s="12"/>
+      <c r="AR17" s="19"/>
+      <c r="AS17" s="19"/>
       <c r="AT17" s="12"/>
-      <c r="AU17" s="12"/>
-      <c r="AV17" s="12"/>
+      <c r="AU17" s="19"/>
+      <c r="AV17" s="19"/>
       <c r="AW17" s="12"/>
       <c r="AX17" s="12"/>
       <c r="AY17" s="12"/>
@@ -2334,11 +2356,11 @@
       <c r="AO18" s="12"/>
       <c r="AP18" s="12"/>
       <c r="AQ18" s="12"/>
-      <c r="AR18" s="12"/>
-      <c r="AS18" s="12"/>
+      <c r="AR18" s="19"/>
+      <c r="AS18" s="19"/>
       <c r="AT18" s="12"/>
-      <c r="AU18" s="12"/>
-      <c r="AV18" s="12"/>
+      <c r="AU18" s="19"/>
+      <c r="AV18" s="19"/>
       <c r="AW18" s="12"/>
       <c r="AX18" s="12"/>
       <c r="AY18" s="12"/>
@@ -2399,11 +2421,11 @@
       <c r="AO19" s="12"/>
       <c r="AP19" s="12"/>
       <c r="AQ19" s="12"/>
-      <c r="AR19" s="12"/>
-      <c r="AS19" s="12"/>
+      <c r="AR19" s="19"/>
+      <c r="AS19" s="19"/>
       <c r="AT19" s="12"/>
-      <c r="AU19" s="12"/>
-      <c r="AV19" s="12"/>
+      <c r="AU19" s="19"/>
+      <c r="AV19" s="19"/>
       <c r="AW19" s="12"/>
       <c r="AX19" s="12"/>
       <c r="AY19" s="12"/>
@@ -2464,11 +2486,11 @@
       <c r="AO20" s="12"/>
       <c r="AP20" s="12"/>
       <c r="AQ20" s="12"/>
-      <c r="AR20" s="12"/>
-      <c r="AS20" s="12"/>
+      <c r="AR20" s="19"/>
+      <c r="AS20" s="19"/>
       <c r="AT20" s="12"/>
-      <c r="AU20" s="12"/>
-      <c r="AV20" s="12"/>
+      <c r="AU20" s="19"/>
+      <c r="AV20" s="19"/>
       <c r="AW20" s="12"/>
       <c r="AX20" s="12"/>
       <c r="AY20" s="12"/>
@@ -2529,11 +2551,11 @@
       <c r="AO21" s="12"/>
       <c r="AP21" s="12"/>
       <c r="AQ21" s="12"/>
-      <c r="AR21" s="12"/>
-      <c r="AS21" s="12"/>
+      <c r="AR21" s="19"/>
+      <c r="AS21" s="19"/>
       <c r="AT21" s="12"/>
-      <c r="AU21" s="12"/>
-      <c r="AV21" s="12"/>
+      <c r="AU21" s="19"/>
+      <c r="AV21" s="19"/>
       <c r="AW21" s="12"/>
       <c r="AX21" s="12"/>
       <c r="AY21" s="12"/>
@@ -2594,11 +2616,11 @@
       <c r="AO22" s="12"/>
       <c r="AP22" s="12"/>
       <c r="AQ22" s="12"/>
-      <c r="AR22" s="12"/>
-      <c r="AS22" s="12"/>
+      <c r="AR22" s="19"/>
+      <c r="AS22" s="19"/>
       <c r="AT22" s="12"/>
-      <c r="AU22" s="12"/>
-      <c r="AV22" s="12"/>
+      <c r="AU22" s="19"/>
+      <c r="AV22" s="19"/>
       <c r="AW22" s="12"/>
       <c r="AX22" s="12"/>
       <c r="AY22" s="12"/>
@@ -2659,11 +2681,11 @@
       <c r="AO23" s="12"/>
       <c r="AP23" s="12"/>
       <c r="AQ23" s="12"/>
-      <c r="AR23" s="12"/>
-      <c r="AS23" s="12"/>
+      <c r="AR23" s="19"/>
+      <c r="AS23" s="19"/>
       <c r="AT23" s="12"/>
-      <c r="AU23" s="12"/>
-      <c r="AV23" s="12"/>
+      <c r="AU23" s="19"/>
+      <c r="AV23" s="19"/>
       <c r="AW23" s="12"/>
       <c r="AX23" s="12"/>
       <c r="AY23" s="12"/>
@@ -2724,11 +2746,11 @@
       <c r="AO24" s="12"/>
       <c r="AP24" s="12"/>
       <c r="AQ24" s="12"/>
-      <c r="AR24" s="12"/>
-      <c r="AS24" s="12"/>
+      <c r="AR24" s="19"/>
+      <c r="AS24" s="19"/>
       <c r="AT24" s="12"/>
-      <c r="AU24" s="12"/>
-      <c r="AV24" s="12"/>
+      <c r="AU24" s="19"/>
+      <c r="AV24" s="19"/>
       <c r="AW24" s="12"/>
       <c r="AX24" s="12"/>
       <c r="AY24" s="12"/>
@@ -2789,11 +2811,11 @@
       <c r="AO25" s="12"/>
       <c r="AP25" s="12"/>
       <c r="AQ25" s="12"/>
-      <c r="AR25" s="12"/>
-      <c r="AS25" s="12"/>
+      <c r="AR25" s="19"/>
+      <c r="AS25" s="19"/>
       <c r="AT25" s="12"/>
-      <c r="AU25" s="12"/>
-      <c r="AV25" s="12"/>
+      <c r="AU25" s="19"/>
+      <c r="AV25" s="19"/>
       <c r="AW25" s="12"/>
       <c r="AX25" s="12"/>
       <c r="AY25" s="12"/>
@@ -2854,11 +2876,11 @@
       <c r="AO26" s="12"/>
       <c r="AP26" s="12"/>
       <c r="AQ26" s="12"/>
-      <c r="AR26" s="12"/>
-      <c r="AS26" s="12"/>
+      <c r="AR26" s="19"/>
+      <c r="AS26" s="19"/>
       <c r="AT26" s="12"/>
-      <c r="AU26" s="12"/>
-      <c r="AV26" s="12"/>
+      <c r="AU26" s="19"/>
+      <c r="AV26" s="19"/>
       <c r="AW26" s="12"/>
       <c r="AX26" s="12"/>
       <c r="AY26" s="12"/>
@@ -2919,11 +2941,11 @@
       <c r="AO27" s="12"/>
       <c r="AP27" s="12"/>
       <c r="AQ27" s="12"/>
-      <c r="AR27" s="12"/>
-      <c r="AS27" s="12"/>
+      <c r="AR27" s="19"/>
+      <c r="AS27" s="19"/>
       <c r="AT27" s="12"/>
-      <c r="AU27" s="12"/>
-      <c r="AV27" s="12"/>
+      <c r="AU27" s="19"/>
+      <c r="AV27" s="19"/>
       <c r="AW27" s="12"/>
       <c r="AX27" s="12"/>
       <c r="AY27" s="12"/>
@@ -2984,11 +3006,11 @@
       <c r="AO28" s="12"/>
       <c r="AP28" s="12"/>
       <c r="AQ28" s="12"/>
-      <c r="AR28" s="12"/>
-      <c r="AS28" s="12"/>
+      <c r="AR28" s="19"/>
+      <c r="AS28" s="19"/>
       <c r="AT28" s="12"/>
-      <c r="AU28" s="12"/>
-      <c r="AV28" s="12"/>
+      <c r="AU28" s="19"/>
+      <c r="AV28" s="19"/>
       <c r="AW28" s="12"/>
       <c r="AX28" s="12"/>
       <c r="AY28" s="12"/>
@@ -3049,11 +3071,11 @@
       <c r="AO29" s="13"/>
       <c r="AP29" s="13"/>
       <c r="AQ29" s="13"/>
-      <c r="AR29" s="13"/>
-      <c r="AS29" s="13"/>
+      <c r="AR29" s="19"/>
+      <c r="AS29" s="19"/>
       <c r="AT29" s="13"/>
-      <c r="AU29" s="13"/>
-      <c r="AV29" s="13"/>
+      <c r="AU29" s="19"/>
+      <c r="AV29" s="19"/>
       <c r="AW29" s="13"/>
       <c r="AX29" s="13"/>
       <c r="AY29" s="13"/>

</xml_diff>